<commit_message>
Update BOM: in-stock caps, fuse holder, new DigiKey cart
Co-authored-by: NikitaBang <NikitaBang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/03-BOM/Purchase_Request_DigiKey_Nikita_Bangiyev_60.xlsx
+++ b/docs/03-BOM/Purchase_Request_DigiKey_Nikita_Bangiyev_60.xlsx
@@ -1684,12 +1684,12 @@
       </c>
       <c r="B15" s="114" t="inlineStr">
         <is>
-          <t>486-1259-ND</t>
+          <t>486-1258-ND</t>
         </is>
       </c>
       <c r="C15" s="109" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=0031.8201</t>
+          <t>https://www.digikey.com/en/products/detail/schurter-inc/0031-8201/669925</t>
         </is>
       </c>
       <c r="D15" s="100" t="n"/>
@@ -2192,17 +2192,17 @@
       </c>
       <c r="B30" s="107" t="inlineStr">
         <is>
-          <t>399-ESK106M016AC3AA-ND</t>
+          <t>399-ESK106M025AC3AA-ND</t>
         </is>
       </c>
       <c r="C30" s="107" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=ESK106M016AC3AA</t>
+          <t>https://www.digikey.com/en/products/detail/kemet/ESK106M025AC3AA/18167956</t>
         </is>
       </c>
       <c r="E30" s="109" t="inlineStr">
         <is>
-          <t>Cap 10uF 16V aluminum radial</t>
+          <t>Cap 10uF 25V aluminum radial</t>
         </is>
       </c>
       <c r="F30" s="100" t="n"/>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="H30" s="110" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="I30" s="111">
         <f>A30*H30</f>
@@ -2225,17 +2225,17 @@
       </c>
       <c r="B31" s="107" t="inlineStr">
         <is>
-          <t>399-T350E106K016AT-ND</t>
+          <t>478-1839-ND</t>
         </is>
       </c>
       <c r="C31" s="107" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/result?keywords=T350E106K016AT</t>
+          <t>https://www.digikey.com/en/products/detail/kyocera-avx/TAP106K016SCS/563942</t>
         </is>
       </c>
       <c r="E31" s="109" t="inlineStr">
         <is>
-          <t>Cap 10uF 16V tantalum radial</t>
+          <t>Cap 10uF 16V tantalum radial (KYOCERA AVX TAP106K016SCS)</t>
         </is>
       </c>
       <c r="F31" s="100" t="n"/>
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="H31" s="110" t="n">
-        <v>4.1</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I31" s="111">
         <f>A31*H31</f>
@@ -2460,77 +2460,77 @@
     </row>
   </sheetData>
   <mergeCells count="71">
+    <mergeCell ref="E12:F12"/>
     <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C24:D24"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="A46:C46"/>
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A40:H40"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E24:F24"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E8:F8"/>
     <mergeCell ref="B43:I43"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C29:D29"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="H46:I46"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="D4:F4"/>
     <mergeCell ref="E28:F28"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C22:D22"/>
     <mergeCell ref="A37:H37"/>
+    <mergeCell ref="C31:D31"/>
     <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C12:D12"/>
     <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="D5:F5"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E2:I2"/>
     <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E27:F27"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C23:D23"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="C8:D8"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="A45:C45"/>
+    <mergeCell ref="E7:F7"/>
     <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="C19:D19"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="C13:D13"/>
+    <mergeCell ref="A6:I6"/>
     <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="E21:F21"/>
+    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" display="https://www.digikey.com/en/products/detail/ams-osram-usa-inc./SFH%25203310/2182181?utm_adgroup=&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=PMax%20Shopping_Product_High%20ROAS%20Categories&amp;utm_term=&amp;utm_content=&amp;utm_id=go_cmp-20222717502_adg-_ad-__dev-c_ext-_prd-2182181_sig-Cj0KCQjwyL24BhCtARIsALo0fSDiVY71lJxIWMS5LDMaQjqT36mUuK9vrlFvG9tfNZNDLtDfc2q5tPUaAr0ZEALw_wcB&amp;gad_source=1&amp;gclid=Cj0KCQjwyL24BhCtARIsALo0fSDiVY71lJxIWMS5LDMaQjqT36mUuK9vrlFvG9tfNZNDLtDfc2q5tPUaAr0ZEALw_wcB" r:id="rId1"/>

</xml_diff>